<commit_message>
Align pre-discount (82%) and post-discount (73%) MNT-Halan market-cap figures across docx and xlsx
Both the Word study and the Excel model previously cited only one of these two
figures at different points -- the docx said '73%' (net of the 10% complexity
discount), the xlsx's SOTP sheet said '82%' (gross, pre-discount). Both were
correct, just different legitimate framings of the same fact, but they didn't
match word-for-word if read side by side.

Now both documents state both figures explicitly everywhere the stat appears:
headline, the MNT-Halan detail table, the plain-terms paragraph, the §1.7 crux,
the §4 verdict, the §7 caveat, and Expert 3's dialogue in the docx; the SOTP
sheet's market-implied-read note in the xlsx. build_xlsx4.py updated to match
so the script/file reconciliation (0 diffs, verified) still holds.
</commit_message>
<xml_diff>
--- a/engine/gbco_study/GBCO_Valuation_Model_08072026_public.xlsx
+++ b/engine/gbco_study/GBCO_Valuation_Model_08072026_public.xlsx
@@ -547,7 +547,7 @@
     <t xml:space="preserve">memo: MNT-Halan per share, post-discount (EGP)</t>
   </si>
   <si>
-    <t xml:space="preserve">The market-implied read is now a genuine puzzle, not a sanity check: mkt cap − lender − associates at the confirmed 41.61% stake implies a NEGATIVE value for the Auto leg (≈ −EGP 3.6bn) — impossible for a real, profitable business. MNT-Halan alone is ≈82% of GB Corp's market cap. Either the market discounts this private mark far more steeply than this study's 10%, or GB Corp is meaningfully mispriced (see the study's §7).</t>
+    <t xml:space="preserve">The market-implied read is now a genuine puzzle, not a sanity check: mkt cap − lender − associates at the confirmed 41.61% stake implies a NEGATIVE value for the Auto leg (≈ −EGP 3.6bn) — impossible for a real, profitable business. MNT-Halan alone is ≈82% of GB Corp's market cap pre-discount (≈73% after this study's 10% complexity discount). Either the market discounts this private mark far more steeply than this study's 10%, or GB Corp is meaningfully mispriced (see the study's §7).</t>
   </si>
   <si>
     <t xml:space="preserve">MNT-Halan stake sensitivity — now largely resolved: 41.61% is a confirmed, dated figure (9-Jun-2026)</t>
@@ -1341,151 +1341,151 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>